<commit_message>
Cambios logic para hacer pruebas, excel y el docs
</commit_message>
<xml_diff>
--- a/Docs/TablasDatos-Lab6.xlsx
+++ b/Docs/TablasDatos-Lab6.xlsx
@@ -1,21 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Universidad\2025-2\Asistencia\Laboratorios\Lab6\ISIS1225-Laboratorio-6\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/j_mujicad_uniandes_edu_co/Documents/2026-2/EDA/Laboratorios/Laboratorio6-G03/Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD33DA02-4501-4B58-9D83-E0FFBD1B4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{FD33DA02-4501-4B58-9D83-E0FFBD1B4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D3920ED-BB10-40A9-896E-6C8FB5B1715C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Lab6" sheetId="1" r:id="rId1"/>
-    <sheet name="Graf Mem Vs Tiempo" sheetId="17" r:id="rId2"/>
-    <sheet name="Graf LF Vs Mem" sheetId="15" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -169,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -203,6 +201,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,7 +456,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -626,6 +627,18 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>724193.76</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>425875.13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>404349.61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>393285.16</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -635,13 +648,25 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>8563.34</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7417.55</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6574.28</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7100.05</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-A503-4D66-A171-A692504BE170}"/>
+              <c16:uniqueId val="{00000001-B02B-405A-A35D-3E409978DCE7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -733,6 +758,18 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>409415.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>401309.96</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>398060.24</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>395228.3</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -742,13 +779,25 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>5106.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6025.89</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8109.26</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6330.62</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-A503-4D66-A171-A692504BE170}"/>
+              <c16:uniqueId val="{00000003-B02B-405A-A35D-3E409978DCE7}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -839,7 +888,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1073,13 +1122,18 @@
       <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1299,13 +1353,25 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0" formatCode="General">
+                  <c:v>724193.76</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>425875.13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>404349.61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>393285.16</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-CF3A-447E-BC9B-881B276C6AE9}"/>
+              <c16:uniqueId val="{00000001-BBCE-40E1-AAF8-D3487014ED84}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1445,13 +1511,25 @@
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>409415.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>401309.96</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>398060.24</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>395228.3</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-CF3A-447E-BC9B-881B276C6AE9}"/>
+              <c16:uniqueId val="{00000003-BBCE-40E1-AAF8-D3487014ED84}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1645,7 +1723,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1747,6 +1825,11 @@
       <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
 </c:chartSpace>
 </file>
 
@@ -2819,39 +2902,31 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{CAFD5B44-21B9-42C7-B503-C146EF1BA3EE}">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
-<file path=xl/chartsheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{680E7371-595A-4F03-ABE3-E0257A96E5F2}">
-  <sheetPr/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</chartsheet>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>623886</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>1587</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>-1</xdr:colOff>
+      <xdr:row>43</xdr:row>
+      <xdr:rowOff>19842</xdr:rowOff>
+    </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDC983B3-B9E2-99DC-EE8B-D0436D555128}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C83D612F-8717-02A9-6571-AFAA5FFD9985}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks noGrp="1"/>
-        </xdr:cNvGraphicFramePr>
+        <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -2864,27 +2939,30 @@
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:absoluteAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:absoluteAnchor>
-    <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="9297051" cy="6073205"/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>40294</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>457387</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>153203</xdr:rowOff>
+    </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E18504E8-A7EA-BD64-3B60-74FDBEF88E11}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BC2377B-DF17-6354-FA30-51CA886074C0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr>
-          <a:graphicFrameLocks noGrp="1"/>
-        </xdr:cNvGraphicFramePr>
+        <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -2892,12 +2970,12 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
     <xdr:clientData/>
-  </xdr:absoluteAnchor>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3223,21 +3301,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5B14742-4EBB-4241-AC8A-0E5F24F7BB7B}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.7265625" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.1796875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
     </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3248,42 +3326,58 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>0.1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="7"/>
+      <c r="B3" s="12">
+        <v>724193.76</v>
+      </c>
+      <c r="C3" s="7">
+        <v>8563.34</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="9">
         <v>0.5</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="7"/>
+      <c r="B4" s="2">
+        <v>425875.13</v>
+      </c>
+      <c r="C4" s="7">
+        <v>7417.55</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>0.7</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7"/>
+      <c r="B5" s="2">
+        <v>404349.61</v>
+      </c>
+      <c r="C5" s="7">
+        <v>6574.28</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="10">
         <v>0.9</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7"/>
+      <c r="B6" s="2">
+        <v>393285.16</v>
+      </c>
+      <c r="C6" s="7">
+        <v>7100.05</v>
+      </c>
     </row>
-    <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="18.5" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
     </row>
-    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -3294,57 +3388,72 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>2</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="5"/>
+      <c r="B11" s="2">
+        <v>409415.8</v>
+      </c>
+      <c r="C11" s="5">
+        <v>5106.29</v>
+      </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>4</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="2">
+        <v>401309.96</v>
+      </c>
+      <c r="C12" s="2">
+        <v>6025.89</v>
+      </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>6</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="B13" s="2">
+        <v>398060.24</v>
+      </c>
+      <c r="C13" s="2">
+        <v>8109.26</v>
+      </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>8</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="2">
+        <v>395228.3</v>
+      </c>
+      <c r="C14" s="2">
+        <v>6330.62</v>
+      </c>
     </row>
-    <row r="23" ht="14.65" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="14.65" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A9:C9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3597,21 +3706,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3636,9 +3744,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>